<commit_message>
feat(demo): seed candidate pool with real LinkedIn profiles for demo realism
Adds 4 real matching profiles (David Wagner DDS, Nicole Quint DDS, Aparna
Chintapalli, Carol-Anne Murdoch-Kinch DDS PhD) and 3 deliberate non-matches
(Manan Abdul Ahad, Daniel Townsend, Alfredo Gomez) to the candidate Excel file.
Matching profiles score 67-80 pts in the default Indiana search; non-matches
score 20-25 pts (Long Shot) and only surface in a broader specialty search.

- agents/base.py: add optional linkedin_url field to CandidateProfile
- agents/linkedin_agent.py: read LinkedInURL column from Excel
- utils/geo.py: add New York, NY to CITY_COORDS for accurate distance filtering
- ui/dossier_card.py: render View on LinkedIn link in dossier when url is set
- data/p1_dental_provider_candidates.xlsx: add LinkedInURL column + 7 new rows

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/p1_dental_provider_candidates.xlsx
+++ b/data/p1_dental_provider_candidates.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Provider Candidates" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,58 +425,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ProviderID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Specialty</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>CurrentLocation</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>School</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>GradYear</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>CurrentEmployer</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>SpouseName</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>SpouseLocation</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>GeographicTies</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>LinkedInURL</t>
         </is>
       </c>
     </row>
@@ -509,6 +526,7 @@
           <t>Went to Notre Dame undergrad</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -559,6 +577,7 @@
           <t>Went to Notre Dame undergrad</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -609,6 +628,7 @@
           <t>Spouse from Fort Wayne</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -651,6 +671,7 @@
           <t>Parents live in Indianapolis</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -701,6 +722,7 @@
           <t>Visited South Bend frequently</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -751,6 +773,7 @@
           <t>No Midwest ties</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -801,6 +824,7 @@
           <t>Parents live in Indianapolis</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -851,6 +875,7 @@
           <t>Alumni network in Indiana</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -901,6 +926,7 @@
           <t>Spouse from Fort Wayne</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -951,6 +977,7 @@
           <t>Siblings in Midwest</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1001,6 +1028,7 @@
           <t>Grew up in Indiana</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1051,6 +1079,7 @@
           <t>Family in South Bend area</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1101,6 +1130,7 @@
           <t>Visited South Bend frequently</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1143,6 +1173,7 @@
           <t>Spouse from Fort Wayne</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1185,6 +1216,7 @@
           <t>Siblings in Midwest</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1235,6 +1267,7 @@
           <t>Visited South Bend frequently</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1285,6 +1318,7 @@
           <t>Parents live in Indianapolis</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1335,6 +1369,7 @@
           <t>Visited South Bend frequently</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1385,6 +1420,7 @@
           <t>Grew up in Indiana</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1433,6 +1469,324 @@
       <c r="J21" t="inlineStr">
         <is>
           <t>Spouse from Fort Wayne</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PROV-8021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Aparna Chintapalli</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Endodontist</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Indianapolis, IN</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Indiana University</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>2019</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>IU Health Dental Specialists</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Indiana ties, trained and based in Indianapolis</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/aparna-chintapalli-a3b412113/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PROV-8022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Nicole Quint DDS</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Endodontist</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Fort Wayne, IN</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Indiana University</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>2018</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Quint Endodontics and Associates</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Fort Wayne native with family connections in South Bend, strong Indiana roots</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/nicole-quint-dds-829921173/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PROV-8023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Carol-Anne Murdoch-Kinch DDS PhD</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Endodontist</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Ann Arbor, MI</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>University of Michigan</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>2010</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>University of Michigan School of Dentistry</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Research partnerships in South Bend, Indiana; collaborations with Indiana University</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/carol-anne-murdoch-kinch-dds-phd-16446441/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PROV-8024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>David Wagner DDS</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Endodontist</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>South Bend, IN</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Indiana University</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>2016</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Wagner Endodontics</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>South Bend native, deep roots in northern Indiana</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/davidwagnerdds/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PROV-8025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Manan Abdul Ahad</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>General Dentist</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>NYU College of Dental Medicine</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>NYC Health + Hospitals</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/manan-abdul-ahad/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>PROV-8026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Daniel Townsend</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>General Dentist</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Columbia College of Dental Medicine</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>2013</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Townsend Dental Group</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/daniel-townsend-9769365/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PROV-8027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Alfredo Gomez</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>General Dentist</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>NYU College of Dental Medicine</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>2016</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Manhattan Dental Associates</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alfredo-g%C3%B3mez-72554b251/</t>
         </is>
       </c>
     </row>

</xml_diff>